<commit_message>
Add writer layer, guards, demo fixtures and the read-only MCP connector
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HzG3VB7cjMR9Rvuy5zCNo7
</commit_message>
<xml_diff>
--- a/data/production/production_2026-W36.xlsx
+++ b/data/production/production_2026-W36.xlsx
@@ -423,7 +423,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G41"/>
+  <dimension ref="A1:G33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -483,31 +483,31 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Aisha Bello</t>
+          <t>Luis Ortega</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>AU-680238</t>
+          <t>HO-957873</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Victor Petrov</t>
+          <t>Grace Albright</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Auto</t>
+          <t>Home</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>New</t>
+          <t>Renewal</t>
         </is>
       </c>
       <c r="G4" t="n">
-        <v>968.27</v>
+        <v>2913.25</v>
       </c>
     </row>
     <row r="5">
@@ -516,22 +516,22 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Aisha Bello</t>
+          <t xml:space="preserve"> Priya Raman</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>HO-488571</t>
+          <t>CM-947206</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Leah Okafor</t>
+          <t>Caleb Whitfield</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Home</t>
+          <t>Commercial</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -540,7 +540,7 @@
         </is>
       </c>
       <c r="G5" t="n">
-        <v>2133.83</v>
+        <v>8417.77</v>
       </c>
     </row>
     <row r="6">
@@ -549,55 +549,55 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Grant Fowler</t>
+          <t>Tom Becker</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>AU-259097</t>
+          <t>HO-100224</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Maria Novak</t>
+          <t>Grace Albright</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Auto</t>
+          <t>Home</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>New</t>
+          <t>Renewal</t>
         </is>
       </c>
       <c r="G6" t="n">
-        <v>1011.12</v>
+        <v>1188.19</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
-        <v>46265</v>
+        <v>46266</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Maya Chen</t>
+          <t>Aisha Bello</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>HO-887443</t>
+          <t>AU-147434</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Alma Ashby</t>
+          <t>Zoe Marsh</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Home</t>
+          <t>Auto</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -606,59 +606,29 @@
         </is>
       </c>
       <c r="G7" t="n">
-        <v>1612.37</v>
+        <v>1870.85</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="2" t="n">
-        <v>46265</v>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>Tom Becker</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>HO-915573</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>Olivia Delgado</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>Home</t>
-        </is>
-      </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>New</t>
-        </is>
-      </c>
-      <c r="G8" t="n">
-        <v>3123.84</v>
-      </c>
+      <c r="A8" s="2" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
-        <v>46265</v>
+        <v>46266</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Tom Becker</t>
+          <t>Aisha Bello</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>LF-427110</t>
+          <t>LF-607343</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Jonah Calloway</t>
+          <t>James Whitfield</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -668,11 +638,11 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>NEW</t>
+          <t>New</t>
         </is>
       </c>
       <c r="G9" t="n">
-        <v>805.39</v>
+        <v>691.5599999999999</v>
       </c>
     </row>
     <row r="10">
@@ -681,165 +651,163 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Aisha Bello</t>
+          <t>Grant Fowler</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>LF-479781</t>
+          <t>AU-749037</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Owen Petrov</t>
+          <t>Ruby Ferreira</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Life</t>
+          <t>Auto</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Renewal</t>
-        </is>
-      </c>
-      <c r="G10" t="inlineStr">
-        <is>
-          <t>$876.01</t>
-        </is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="G10" t="n">
+        <v>2395.7</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
-        <v>46266</v>
+        <v>46267</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Luis Ortega</t>
+          <t>Aisha Bello</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>AU-245095</t>
+          <t>HO-296292</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Olivia Hartley</t>
+          <t>Maria Ashby</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Auto</t>
+          <t>Home</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Renewal</t>
+          <t>New</t>
         </is>
       </c>
       <c r="G11" t="n">
-        <v>1757.18</v>
+        <v>1265.18</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="n">
-        <v>46266</v>
+        <v>46267</v>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Maya Chen</t>
+          <t xml:space="preserve">Aisha Bello </t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>AU-749342</t>
+          <t>HO-546016</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Maria Duarte</t>
+          <t>Zoe Marsh</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Auto</t>
+          <t xml:space="preserve">Home </t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Renewal</t>
+          <t>New</t>
         </is>
       </c>
       <c r="G12" t="n">
-        <v>2071.64</v>
+        <v>1490.61</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="n">
-        <v>46266</v>
+        <v>46267</v>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Maya Chen</t>
+          <t>Grant Fowler</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>HO-932291</t>
+          <t>LF-307039</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Theo Moreau</t>
+          <t>Marcus Novak</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Home</t>
+          <t>Life</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Renewal</t>
+          <t>New</t>
         </is>
       </c>
       <c r="G13" t="n">
-        <v>2367.79</v>
+        <v>1630.1</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="n">
-        <v>46266</v>
+        <v>46267</v>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Tom Becker</t>
+          <t>Maya Chen</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>LF-309044</t>
+          <t>AU-944246</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Caleb Whitfield</t>
+          <t>Ivy Hartley</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Life</t>
+          <t>Auto</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Renewal</t>
+          <t>New</t>
         </is>
       </c>
       <c r="G14" t="n">
-        <v>2556.21</v>
+        <v>1277.27</v>
       </c>
     </row>
     <row r="15">
@@ -848,31 +816,31 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Aisha Bello</t>
+          <t>Maya Chen</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>AU-745830</t>
+          <t>HO-351589</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Felix Lindqvist</t>
+          <t>Owen Kowal</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Auto</t>
+          <t>Home</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>New</t>
+          <t>Renewal</t>
         </is>
       </c>
       <c r="G15" t="n">
-        <v>1682.62</v>
+        <v>2289.97</v>
       </c>
     </row>
     <row r="16">
@@ -881,22 +849,22 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Aisha Bello</t>
+          <t>Tom Becker</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>LF-993085</t>
+          <t>LF-262278</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Felix Tanaka</t>
+          <t>Maria Lopez</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Life</t>
+          <t>LIFE</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -905,45 +873,45 @@
         </is>
       </c>
       <c r="G16" t="n">
-        <v>1725.7</v>
+        <v>1870.11</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="n">
-        <v>46267</v>
+        <v>46268</v>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Luis Ortega</t>
+          <t>Grant Fowler</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>AU-561239</t>
+          <t>CM-434372</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Mila Tanaka</t>
+          <t>Owen Petrov</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Auto</t>
+          <t>Commercial</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Renewal</t>
+          <t>New</t>
         </is>
       </c>
       <c r="G17" t="n">
-        <v>1275.06</v>
+        <v>3295.05</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="n">
-        <v>46267</v>
+        <v>46268</v>
       </c>
       <c r="B18" t="inlineStr">
         <is>
@@ -952,12 +920,12 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>AU-890075</t>
+          <t>AU-340047</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Zoe Marsh</t>
+          <t>Victor Castillo</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -967,82 +935,82 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>New</t>
+          <t>Renewal</t>
         </is>
       </c>
       <c r="G18" t="n">
-        <v>2314.11</v>
+        <v>1100.59</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="n">
-        <v>46267</v>
+        <v>46268</v>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t xml:space="preserve">Luis Ortega </t>
+          <t>Luis Ortega</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>LF-597732</t>
+          <t>HO-554103</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Leah Novak</t>
+          <t>Grace Delgado</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Life</t>
+          <t>Home</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Renewal</t>
+          <t>New</t>
         </is>
       </c>
       <c r="G19" t="n">
-        <v>2179.55</v>
+        <v>2790.28</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="n">
-        <v>46267</v>
+        <v>46268</v>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Priya Raman</t>
+          <t>Maya Chen</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>CM-372793</t>
+          <t>LF-691396</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Mila Tanaka</t>
+          <t>Victor Castillo</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Commercial</t>
+          <t>Life</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>Renewal</t>
+          <t>New</t>
         </is>
       </c>
       <c r="G20" t="n">
-        <v>3687.68</v>
+        <v>1091.42</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="n">
-        <v>46267</v>
+        <v>46268</v>
       </c>
       <c r="B21" t="inlineStr">
         <is>
@@ -1051,12 +1019,12 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>CM-593152</t>
+          <t>CM-477420</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Ivy Hartley</t>
+          <t>Maria Duarte</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -1070,12 +1038,12 @@
         </is>
       </c>
       <c r="G21" t="n">
-        <v>8330.5</v>
+        <v>8602.1</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="n">
-        <v>46267</v>
+        <v>46268</v>
       </c>
       <c r="B22" t="inlineStr">
         <is>
@@ -1084,26 +1052,26 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>HO-328552</t>
+          <t>AU-823262</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Olivia Delgado</t>
+          <t>Marcus Okafor</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Home</t>
+          <t>Auto</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>Renewal</t>
+          <t>New</t>
         </is>
       </c>
       <c r="G22" t="n">
-        <v>1351.53</v>
+        <v>1774.6</v>
       </c>
     </row>
     <row r="23">
@@ -1112,53 +1080,83 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Aisha Bello</t>
+          <t>Tom Becker</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>LF-355709</t>
+          <t>HO-488108</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Grace Albright</t>
+          <t>Elena Novak</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
+          <t>Home</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>Renewal</t>
+        </is>
+      </c>
+      <c r="G23" t="n">
+        <v>3242.99</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="n">
+        <v>46268</v>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Tom Becker</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>LF-443681</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Maria Novak</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
           <t>Life</t>
         </is>
       </c>
-      <c r="F23" t="inlineStr">
+      <c r="F24" t="inlineStr">
         <is>
           <t>New</t>
         </is>
       </c>
-      <c r="G23" t="n">
-        <v>764.66</v>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="2" t="n"/>
+      <c r="G24" t="n">
+        <v>648.61</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="n">
-        <v>46268</v>
+        <v>46269</v>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Grant Fowler</t>
+          <t>Aisha Bello</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>AU-564226</t>
+          <t>AU-244411</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Maria Duarte</t>
+          <t>Ivy Okafor</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
@@ -1173,27 +1171,27 @@
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>$1,683.86</t>
+          <t>$1,694.90</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="n">
-        <v>46268</v>
+        <v>46269</v>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>GRANT FOWLER</t>
+          <t>Aisha Bello</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>HO-457256</t>
+          <t>HO-727278</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Ruby Sorensen</t>
+          <t>Felix Tanaka</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
@@ -1203,51 +1201,51 @@
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>New</t>
+          <t>Renewal</t>
         </is>
       </c>
       <c r="G26" t="n">
-        <v>2085.73</v>
+        <v>1944.91</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="n">
-        <v>46268</v>
+        <v>46269</v>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Grant Fowler</t>
+          <t>Aisha Bello</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>LF-219629</t>
+          <t>HO-748655</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Adrian Okafor</t>
+          <t>Samuel Brennan</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Life</t>
+          <t>Home</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>New</t>
+          <t>Renewal</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>$1,079.71</t>
+          <t>$2,065.44</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="n">
-        <v>46268</v>
+        <v>46269</v>
       </c>
       <c r="B28" t="inlineStr">
         <is>
@@ -1256,12 +1254,12 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>AU-609232</t>
+          <t>AU-938653</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Maria Moreau</t>
+          <t>Sofia Pryor</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
@@ -1274,13 +1272,15 @@
           <t>New</t>
         </is>
       </c>
-      <c r="G28" t="n">
-        <v>1229.13</v>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>$2,397.33</t>
+        </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="n">
-        <v>46268</v>
+        <v>46269</v>
       </c>
       <c r="B29" t="inlineStr">
         <is>
@@ -1289,31 +1289,31 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>AU-668969</t>
+          <t>HO-363199</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Zoe Marsh</t>
+          <t>Marcus Novak</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Auto</t>
+          <t>home</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>Renewal</t>
+          <t>New</t>
         </is>
       </c>
       <c r="G29" t="n">
-        <v>1480.17</v>
+        <v>3115.21</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="n">
-        <v>46268</v>
+        <v>46269</v>
       </c>
       <c r="B30" t="inlineStr">
         <is>
@@ -1322,78 +1322,78 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>AU-708158</t>
+          <t>CM-751673</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Owen Sorensen</t>
+          <t>Mila Tanaka</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Auto</t>
+          <t>Commercial</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Renewal</t>
+          <t>Renewal</t>
         </is>
       </c>
       <c r="G30" t="n">
-        <v>1573.16</v>
+        <v>9043.969999999999</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="n">
-        <v>46268</v>
+        <v>46269</v>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Maya Chen</t>
+          <t>Priya Raman</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>AU-800005</t>
+          <t>HO-203152</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Leah Novak</t>
+          <t>Alma Ashby</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Auto</t>
+          <t>Home</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>New</t>
+          <t>Renewal</t>
         </is>
       </c>
       <c r="G31" t="n">
-        <v>1100.01</v>
+        <v>3259.69</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="n">
-        <v>46268</v>
+        <v>46269</v>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Maya Chen</t>
+          <t>Tom Becker</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>LF-742412</t>
+          <t>LF-146828</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Marcus Ibsen</t>
+          <t>Zoe Marsh</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
@@ -1407,284 +1407,18 @@
         </is>
       </c>
       <c r="G32" t="n">
-        <v>1731.36</v>
+        <v>1070.89</v>
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="2" t="n">
-        <v>46268</v>
-      </c>
+      <c r="A33" s="2" t="n"/>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Priya Raman</t>
-        </is>
-      </c>
-      <c r="C33" t="inlineStr">
-        <is>
-          <t>CM-720644</t>
-        </is>
-      </c>
-      <c r="D33" t="inlineStr">
-        <is>
-          <t>Caleb Whitfield</t>
-        </is>
-      </c>
-      <c r="E33" t="inlineStr">
-        <is>
-          <t>Commercial</t>
-        </is>
-      </c>
-      <c r="F33" t="inlineStr">
-        <is>
-          <t>Renewal</t>
+          <t>TOTAL</t>
         </is>
       </c>
       <c r="G33" t="n">
-        <v>8177.32</v>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="2" t="n">
-        <v>46268</v>
-      </c>
-      <c r="B34" t="inlineStr">
-        <is>
-          <t>Tom Becker</t>
-        </is>
-      </c>
-      <c r="C34" t="inlineStr">
-        <is>
-          <t>LF-849747</t>
-        </is>
-      </c>
-      <c r="D34" t="inlineStr">
-        <is>
-          <t>Maria Ashby</t>
-        </is>
-      </c>
-      <c r="E34" t="inlineStr">
-        <is>
-          <t>Life</t>
-        </is>
-      </c>
-      <c r="F34" t="inlineStr">
-        <is>
-          <t>New</t>
-        </is>
-      </c>
-      <c r="G34" t="n">
-        <v>2420.53</v>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="2" t="n">
-        <v>46269</v>
-      </c>
-      <c r="B35" t="inlineStr">
-        <is>
-          <t>Aisha Bello</t>
-        </is>
-      </c>
-      <c r="C35" t="inlineStr">
-        <is>
-          <t>AU-991597</t>
-        </is>
-      </c>
-      <c r="D35" t="inlineStr">
-        <is>
-          <t>Grace Delgado</t>
-        </is>
-      </c>
-      <c r="E35" t="inlineStr">
-        <is>
-          <t>Auto</t>
-        </is>
-      </c>
-      <c r="F35" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> Renewal</t>
-        </is>
-      </c>
-      <c r="G35" t="n">
-        <v>2245.71</v>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" s="2" t="n">
-        <v>46269</v>
-      </c>
-      <c r="B36" t="inlineStr">
-        <is>
-          <t>Grant Fowler</t>
-        </is>
-      </c>
-      <c r="C36" t="inlineStr">
-        <is>
-          <t>AU-901577</t>
-        </is>
-      </c>
-      <c r="D36" t="inlineStr">
-        <is>
-          <t>Leah Okafor</t>
-        </is>
-      </c>
-      <c r="E36" t="inlineStr">
-        <is>
-          <t>Auto</t>
-        </is>
-      </c>
-      <c r="F36" t="inlineStr">
-        <is>
-          <t>New</t>
-        </is>
-      </c>
-      <c r="G36" t="n">
-        <v>1272.29</v>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="2" t="n">
-        <v>46269</v>
-      </c>
-      <c r="B37" t="inlineStr">
-        <is>
-          <t>Luis Ortega</t>
-        </is>
-      </c>
-      <c r="C37" t="inlineStr">
-        <is>
-          <t>LF-829308</t>
-        </is>
-      </c>
-      <c r="D37" t="inlineStr">
-        <is>
-          <t>Zoe Marsh</t>
-        </is>
-      </c>
-      <c r="E37" t="inlineStr">
-        <is>
-          <t>Life</t>
-        </is>
-      </c>
-      <c r="F37" t="inlineStr">
-        <is>
-          <t>Renewal</t>
-        </is>
-      </c>
-      <c r="G37" t="n">
-        <v>1884.31</v>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="2" t="n">
-        <v>46269</v>
-      </c>
-      <c r="B38" t="inlineStr">
-        <is>
-          <t>MAYA CHEN</t>
-        </is>
-      </c>
-      <c r="C38" t="inlineStr">
-        <is>
-          <t>AU-125611</t>
-        </is>
-      </c>
-      <c r="D38" t="inlineStr">
-        <is>
-          <t>Adrian Okafor</t>
-        </is>
-      </c>
-      <c r="E38" t="inlineStr">
-        <is>
-          <t>Auto</t>
-        </is>
-      </c>
-      <c r="F38" t="inlineStr">
-        <is>
-          <t>Renewal</t>
-        </is>
-      </c>
-      <c r="G38" t="inlineStr">
-        <is>
-          <t>$1,339.64</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" s="2" t="n">
-        <v>46269</v>
-      </c>
-      <c r="B39" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Maya Chen </t>
-        </is>
-      </c>
-      <c r="C39" t="inlineStr">
-        <is>
-          <t>HO-303880</t>
-        </is>
-      </c>
-      <c r="D39" t="inlineStr">
-        <is>
-          <t>Zoe Marsh</t>
-        </is>
-      </c>
-      <c r="E39" t="inlineStr">
-        <is>
-          <t>Home</t>
-        </is>
-      </c>
-      <c r="F39" t="inlineStr">
-        <is>
-          <t>New</t>
-        </is>
-      </c>
-      <c r="G39" t="n">
-        <v>2960.89</v>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" s="2" t="n">
-        <v>46269</v>
-      </c>
-      <c r="B40" t="inlineStr">
-        <is>
-          <t>Maya Chen</t>
-        </is>
-      </c>
-      <c r="C40" t="inlineStr">
-        <is>
-          <t>HO-587115</t>
-        </is>
-      </c>
-      <c r="D40" t="inlineStr">
-        <is>
-          <t>Samuel Brennan</t>
-        </is>
-      </c>
-      <c r="E40" t="inlineStr">
-        <is>
-          <t>Home</t>
-        </is>
-      </c>
-      <c r="F40" t="inlineStr">
-        <is>
-          <t>New</t>
-        </is>
-      </c>
-      <c r="G40" t="n">
-        <v>1559.57</v>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="2" t="n"/>
-      <c r="B41" t="inlineStr">
-        <is>
-          <t>TOTAL</t>
-        </is>
-      </c>
-      <c r="G41" t="n">
-        <v>76418.45</v>
+        <v>74438.53999999999</v>
       </c>
     </row>
   </sheetData>
@@ -1698,7 +1432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E21"/>
+  <dimension ref="A1:E15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1736,16 +1470,16 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>AU-708158</t>
+          <t>CM-751673</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Auto</t>
+          <t>Commercial</t>
         </is>
       </c>
       <c r="D2" t="n">
-        <v>1544.83</v>
+        <v>8316.25</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
@@ -1761,7 +1495,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>HO-932291</t>
+          <t>HO-351589</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -1770,7 +1504,7 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>2173.47</v>
+        <v>2331.69</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
@@ -1781,21 +1515,21 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Maya Chen</t>
+          <t>Luis Ortega</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>AU-749342</t>
+          <t>HO-957873</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Auto</t>
+          <t>Home</t>
         </is>
       </c>
       <c r="D4" t="n">
-        <v>1895.78</v>
+        <v>2708.24</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
@@ -1806,12 +1540,12 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Maya Chen</t>
+          <t>Luis Ortega</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>AU-125611</t>
+          <t>AU-340047</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -1820,7 +1554,7 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>1198.69</v>
+        <v>1113.62</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
@@ -1831,46 +1565,46 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Luis Ortega</t>
+          <t>Priya Raman</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>LF-597732</t>
+          <t>AU-726286</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Life</t>
+          <t>Auto</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>2012.95</v>
+        <v>1124.77</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Renewed</t>
+          <t>Lost</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Luis Ortega</t>
+          <t>Priya Raman</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>AU-561239</t>
+          <t>CM-477420</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Auto</t>
+          <t>Commercial</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>1258.87</v>
+        <v>8525.23</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -1881,21 +1615,21 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Luis Ortega</t>
+          <t>Priya Raman</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>AU-245095</t>
+          <t>CM-947206</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Auto</t>
+          <t>Commercial</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>1710.23</v>
+        <v>7870.13</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
@@ -1906,21 +1640,21 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Luis Ortega</t>
+          <t>Priya Raman</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>AU-668969</t>
+          <t>HO-203152</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Auto</t>
+          <t>Home</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>1511.4</v>
+        <v>3025.3</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
@@ -1931,12 +1665,12 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Luis Ortega</t>
+          <t>Tom Becker</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>LF-829308</t>
+          <t>LF-602421</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -1945,57 +1679,57 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>1709.75</v>
+        <v>2200.64</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Renewed</t>
+          <t>Lost</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Priya Raman</t>
+          <t>Tom Becker</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>CM-233827</t>
+          <t>HO-488108</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Commercial</t>
+          <t>Home</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>7963.29</v>
+        <v>2996.85</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Lost</t>
+          <t>Renewed</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Priya Raman</t>
+          <t>Tom Becker</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>CM-720644</t>
+          <t>HO-100224</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Commercial</t>
+          <t>Home</t>
         </is>
       </c>
       <c r="D12" t="n">
-        <v>8395.040000000001</v>
+        <v>1129.47</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
@@ -2006,21 +1740,21 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Priya Raman</t>
+          <t>Aisha Bello</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>CM-372793</t>
+          <t>HO-748655</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Commercial</t>
+          <t>Home</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>3681.24</v>
+        <v>2079.82</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
@@ -2031,198 +1765,48 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Priya Raman</t>
+          <t>Aisha Bello</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>CM-888539</t>
+          <t>HO-727278</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Commercial</t>
+          <t>Home</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>4964.32</v>
+        <v>1806.48</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Lost</t>
+          <t>Renewed</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Priya Raman</t>
+          <t>Grant Fowler</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>CM-593152</t>
+          <t>AU-862447</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Commercial</t>
+          <t>Auto</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>7926.92</v>
+        <v>1395.82</v>
       </c>
       <c r="E15" t="inlineStr">
-        <is>
-          <t>Renewed</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>Tom Becker</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>LF-309044</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>Life</t>
-        </is>
-      </c>
-      <c r="D16" t="n">
-        <v>2404.26</v>
-      </c>
-      <c r="E16" t="inlineStr">
-        <is>
-          <t>Renewed</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>Tom Becker</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>HO-328552</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>Home</t>
-        </is>
-      </c>
-      <c r="D17" t="n">
-        <v>1340.22</v>
-      </c>
-      <c r="E17" t="inlineStr">
-        <is>
-          <t>Renewed</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>Aisha Bello</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>AU-991597</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>Auto</t>
-        </is>
-      </c>
-      <c r="D18" t="n">
-        <v>2058.72</v>
-      </c>
-      <c r="E18" t="inlineStr">
-        <is>
-          <t>Renewed</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>Aisha Bello</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>HO-488571</t>
-        </is>
-      </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>Home</t>
-        </is>
-      </c>
-      <c r="D19" t="n">
-        <v>1999.59</v>
-      </c>
-      <c r="E19" t="inlineStr">
-        <is>
-          <t>Renewed</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>Aisha Bello</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>LF-479781</t>
-        </is>
-      </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>Life</t>
-        </is>
-      </c>
-      <c r="D20" t="n">
-        <v>800.52</v>
-      </c>
-      <c r="E20" t="inlineStr">
-        <is>
-          <t>Renewed</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>Grant Fowler</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>HO-207570</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>Home</t>
-        </is>
-      </c>
-      <c r="D21" t="n">
-        <v>2680.86</v>
-      </c>
-      <c r="E21" t="inlineStr">
         <is>
           <t>Lost</t>
         </is>

</xml_diff>